<commit_message>
Tool list 2027 : entièrement en français
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XPwnZBmWUGhvYebrP3X3Z2
</commit_message>
<xml_diff>
--- a/devis_2027/Devis_Enedril_2027_EN.xlsx
+++ b/devis_2027/Devis_Enedril_2027_EN.xlsx
@@ -1988,7 +1988,7 @@
     <row r="32">
       <c r="C32" s="21" t="inlineStr">
         <is>
-          <t>Pour la tool list : copier les colonnes B à D (Bannière, Description, Qté) et les coller dans le classeur « Tool List » (sans les prix).</t>
+          <t>Pour la liste de matériel : copier les colonnes B à D (Bannière, Description, Qté) et les coller dans le classeur « Tool List » (sans les prix).</t>
         </is>
       </c>
     </row>
@@ -5232,7 +5232,7 @@
       </c>
       <c r="J5" s="57" t="inlineStr">
         <is>
-          <t>Loose (vrac)</t>
+          <t>Vrac</t>
         </is>
       </c>
       <c r="K5" s="57" t="inlineStr">
@@ -5331,7 +5331,7 @@
     <row r="12">
       <c r="K12" s="57" t="inlineStr">
         <is>
-          <t>Loose</t>
+          <t>Vrac</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Service ticket : correction de l'affichage des dates (#VALEUR!), opérateurs avec tarif journalier et mob/demob ; devis : dates et montants indépendants de la langue d'Excel
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XPwnZBmWUGhvYebrP3X3Z2
</commit_message>
<xml_diff>
--- a/devis_2027/Devis_Enedril_2027_EN.xlsx
+++ b/devis_2027/Devis_Enedril_2027_EN.xlsx
@@ -2507,7 +2507,7 @@
       <c r="B2" s="1" t="n"/>
       <c r="C2" s="1" t="n"/>
       <c r="D2" s="30">
-        <f>"N° "&amp;'1 Affaire'!$C$6&amp;"   ·   "&amp;IF('1 Affaire'!$C$7="","",TEXT('1 Affaire'!$C$7,"dd/mm/yyyy"))</f>
+        <f>"N° "&amp;'1 Affaire'!$C$6&amp;"   ·   "&amp;IF('1 Affaire'!$C$7="","",TEXT(DAY('1 Affaire'!$C$7),"00")&amp;"/"&amp;TEXT(MONTH('1 Affaire'!$C$7),"00")&amp;"/"&amp;YEAR('1 Affaire'!$C$7))</f>
         <v/>
       </c>
       <c r="K2" s="1" t="n"/>
@@ -2554,7 +2554,7 @@
       <c r="F6" s="33" t="n"/>
       <c r="G6" s="33" t="n"/>
       <c r="H6" s="32">
-        <f>IF('1 Affaire'!$C$7="","",TEXT('1 Affaire'!$C$7,"dd/mm/yyyy"))</f>
+        <f>IF('1 Affaire'!$C$7="","",TEXT(DAY('1 Affaire'!$C$7),"00")&amp;"/"&amp;TEXT(MONTH('1 Affaire'!$C$7),"00")&amp;"/"&amp;YEAR('1 Affaire'!$C$7))</f>
         <v/>
       </c>
       <c r="I6" s="33" t="n"/>
@@ -8120,7 +8120,7 @@
         <v/>
       </c>
       <c r="L34">
-        <f>TEXT('3 Options'!$H$13,"#,##0.00")&amp;" € HT"</f>
+        <f>FIXED('3 Options'!$H$13,2)&amp;" € HT"</f>
         <v/>
       </c>
     </row>

</xml_diff>